<commit_message>
attempt to fix dataset
</commit_message>
<xml_diff>
--- a/rules/CORE-000733/negative/01/data/unit-test-coreid-CG0281-negative.xlsx
+++ b/rules/CORE-000733/negative/01/data/unit-test-coreid-CG0281-negative.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source\core-contributor\rules\CORE-000733\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8BF0FA-7C63-48BE-B4D0-5894E245EF04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E586A89E-D268-42B7-91B0-63B53A06D983}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="42">
   <si>
     <t>Product</t>
   </si>
@@ -136,9 +136,6 @@
     <t>Zanomaline</t>
   </si>
   <si>
-    <t>[ABSENT]</t>
-  </si>
-  <si>
     <t>$randqt_count</t>
   </si>
   <si>
@@ -148,7 +145,10 @@
     <t>TRT</t>
   </si>
   <si>
-    <t>Record</t>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
 </sst>
 </file>
@@ -180,7 +180,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -191,12 +191,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
     <fill>
@@ -233,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -253,13 +247,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -619,7 +610,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -653,16 +644,16 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" t="s">
-        <v>37</v>
+        <v>35</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -676,32 +667,12 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4">
         <v>0</v>
       </c>
     </row>
@@ -728,7 +699,7 @@
       <c r="D1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>18</v>
       </c>
       <c r="F1" s="5" t="s">
@@ -818,22 +789,32 @@
         <v>1</v>
       </c>
       <c r="D5" s="8"/>
-      <c r="E5" s="11" t="s">
-        <v>40</v>
+      <c r="E5" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="9"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="8">
+        <v>1</v>
+      </c>
       <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
+      <c r="E6" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
+      <c r="G6" s="8" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>

</xml_diff>